<commit_message>
📚 Actualización de contenido académico - 2026-03-07 07:38
</commit_message>
<xml_diff>
--- a/04-week/02-session/Book1.xlsx
+++ b/04-week/02-session/Book1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\www\Sena\ADSO-3145555\04-week\01-session\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\www\Sena\ADSO-3145555\04-week\02-session\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15940D7F-D83A-4C7D-B2F9-789807D14B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D126395A-2E0A-4556-A438-6F56D724BA54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{DE9F400F-798B-44FD-824C-C31AA1809054}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{DE9F400F-798B-44FD-824C-C31AA1809054}"/>
   </bookViews>
   <sheets>
     <sheet name="item-1" sheetId="1" r:id="rId1"/>
@@ -99,7 +99,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -109,6 +109,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -125,15 +131,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,7 +505,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B2">
@@ -510,7 +519,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
+      <c r="A3" s="3"/>
       <c r="B3">
         <v>2</v>
       </c>
@@ -522,11 +531,11 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
+      <c r="A4" s="3"/>
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D4" t="s">
@@ -572,13 +581,13 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D2" t="s">
@@ -586,7 +595,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
+      <c r="A3" s="3"/>
       <c r="B3">
         <v>2</v>
       </c>
@@ -598,7 +607,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
+      <c r="A4" s="3"/>
       <c r="B4">
         <v>3</v>
       </c>
@@ -645,7 +654,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B2">
@@ -659,7 +668,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
+      <c r="A3" s="3"/>
       <c r="B3">
         <v>2</v>
       </c>
@@ -671,7 +680,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
+      <c r="A4" s="3"/>
       <c r="B4">
         <v>3</v>
       </c>
@@ -718,7 +727,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B2">
@@ -732,7 +741,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
+      <c r="A3" s="3"/>
       <c r="B3">
         <v>2</v>
       </c>
@@ -744,7 +753,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
+      <c r="A4" s="3"/>
       <c r="B4">
         <v>3</v>
       </c>

</xml_diff>